<commit_message>
Remove hardcoded 3 badge from Calling Campaigns
</commit_message>
<xml_diff>
--- a/backend/candidate_call_results_16612688-3635-4101-a28f-3209733a2249.xlsx
+++ b/backend/candidate_call_results_16612688-3635-4101-a28f-3209733a2249.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N158"/>
+  <dimension ref="A1:N159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12269,6 +12269,87 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>f6dab744-2158-4178-b348-fcee45c04ef2</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>SHIVAM KUMAR</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>shivamkumarsingh2909@gmail.com</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>9877082909</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>2 years</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>interested</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assistant: Hello SHIVAM KUMAR, I'm calling regarding the AI Engineer opportunity at Hireonomous. Is now a good time to talk?
+user:  yes
+assistant:  Are you interested in the AI Engineer opportunity at Hireonomous?
+user:  yes yes
+assistant:  Thanks for confirming. How many years of total work experience do you have?
+user:  total identity year of work experience
+assistant:  Just to clarify, could you please tell me how many years of work experience you have in total?
+user:  three three
+assistant: Got it, you have three years of total work experience. Thank you for sharing that. That concludes my screening questions for now. We'll be in touch regarding the next steps. Have a great day!
+</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>2026-08-31 12:04:22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>